<commit_message>
Cache system: groq+scrape cache, integrated into ai-analysis, sentimen, harga, pertanian
</commit_message>
<xml_diff>
--- a/data/sentimen_berita.xlsx
+++ b/data/sentimen_berita.xlsx
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4982,6 +4982,566 @@
         <v>0</v>
       </c>
       <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>detikFinance - Berita Ekonomi Bisnis, dan Investasi Hari Ini</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>[Purbaya soal Efisiensi Anggaran MBG: Saya Maunya Nol, Tapi Nggak Bisa Kan](https://finance.detik.com/berita-ekonomi-bisnis/d-8549550/purbaya-soal-efisiensi-anggaran-mbg-saya-maunya-nol-tapi-nggak-bisa-kan)</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>[Trump Murka! AS Serang Iran Lagi](https://finance.detik.com/berita-ekonomi-bisnis/d-8549337/trump-murka-as-serang-iran-lagi)</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>[Terungkap Kondisi Pasokan Batu Bara PLN](https://finance.detik.com/energi/d-8549000/terungkap-kondisi-pasokan-batu-bara-pln)</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>[Duit Jumbo dari AIIB China yang Kata Purbaya Bukan Utang](https://finance.detik.com/berita-ekonomi-bisnis/d-8549025/duit-jumbo-dari-aiib-china-yang-kata-purbaya-bukan-utang)</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>[Rute MRT Lebak Bulus-Serpong Masih Rahasia demi Hindari Calo Tanah](https://finance.detik.com/infrastruktur/d-8549184/rute-mrt-lebak-bulus-serpong-masih-rahasia-demi-hindari-calo-tanah)</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>[Stok Batu Bara PLN Aman, ESDM Buka Lagi Keran Ekspor](https://finance.detik.com/energi/d-8549352/stok-batu-bara-pln-aman-esdm-buka-lagi-keran-ekspor)</t>
+        </is>
+      </c>
+      <c r="E133" s="4" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="F133" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G133" s="4" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>[Ekspor Batu Bara Sempat Ditahan demi Pasokan ke PLN](https://finance.detik.com/energi/d-8548667/ekspor-batu-bara-sempat-ditahan-demi-pasokan-ke-pln)</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>[Beras IR. III (IR 64)](https://finance.detik.com/info-pangan/jakarta/beras-ir-iii-ir-64)</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>[Cabe Merah Keriting](https://finance.detik.com/info-pangan/jakarta/cabe-merah-keriting)</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>[Daging Sapi Murni (Semur)](https://finance.detik.com/info-pangan/jakarta/daging-sapi-murni-semur)</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D138" s="5" t="inlineStr">
+        <is>
+          <t>[Beli TV LED 50" UHD Smart di Transmart Full Day Sale Diskonnya Jutaan](https://finance.detik.com/berita-ekonomi-bisnis/d-8549706/beli-tv-led-50-uhd-smart-di-transmart-full-day-sale-diskonnya-jutaan)</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="F138" s="4" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="G138" s="4" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>[Puncak El Nino di Depan Mata, Pemerintah Pede Stok Beras Aman hingga Mei 2027](https://finance.detik.com/berita-ekonomi-bisnis/d-8549545/puncak-el-nino-di-depan-mata-pemerintah-pede-stok-beras-aman-hingga-mei-2027)</t>
+        </is>
+      </c>
+      <c r="E139" s="4" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="F139" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G139" s="4" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>[Transmart Full Day Sale: Harga Sepeda Anak Cuma Rp 1 Jutaan!](https://finance.detik.com/berita-ekonomi-bisnis/d-8549696/transmart-full-day-sale-harga-sepeda-anak-cuma-rp-1-jutaan)</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>[Kemenperin Soroti Penyebab Implementasi Kebijakan HGBT Belum Optimal](https://finance.detik.com/industri/d-8550008/kemenperin-soroti-penyebab-implementasi-kebijakan-hgbt-belum-optimal)</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>Rekomendasi untuk Anda</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
         <is>
           <t>detik finance</t>
         </is>
@@ -5030,7 +5590,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
@@ -5045,11 +5605,11 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
@@ -5064,7 +5624,7 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>17.7%</t>
         </is>
       </c>
     </row>
@@ -5075,11 +5635,11 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>70.4%</t>
+          <t>71.6%</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5650,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>-0.08400000000000001</v>
+        <v>-0.062</v>
       </c>
       <c r="C6" s="8" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Update all data 28/06: sembako, sentimen, pertanian, emas, crypto, bbm, cuaca
</commit_message>
<xml_diff>
--- a/data/sentimen_berita.xlsx
+++ b/data/sentimen_berita.xlsx
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G158"/>
+  <dimension ref="A1:G174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6102,6 +6102,566 @@
         <v>-0.65</v>
       </c>
       <c r="G158" s="6" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>detikFinance - Berita Ekonomi Bisnis, dan Investasi Hari Ini</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B160" s="6" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C160" s="6" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D160" s="7" t="inlineStr">
+        <is>
+          <t>[Harga Emas Antam Turun dalam Sepekan, Buyback Anjlok Rp 20 Ribu/Gram](https://finance.detik.com/berita-ekonomi-bisnis/d-8550494/harga-emas-antam-turun-dalam-sepekan-buyback-anjlok-rp-20-ribu-gram)</t>
+        </is>
+      </c>
+      <c r="E160" s="6" t="inlineStr">
+        <is>
+          <t>NEGATIF</t>
+        </is>
+      </c>
+      <c r="F160" s="6" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="G160" s="6" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B161" s="6" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C161" s="6" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D161" s="7" t="inlineStr">
+        <is>
+          <t>[Harga Ayam di Pasar Ikut Anjlok Jadi Rp 35.000/Kg, Ini Biang Keroknya](https://finance.detik.com/berita-ekonomi-bisnis/d-8550248/harga-ayam-di-pasar-ikut-anjlok-jadi-rp-35-000-kg-ini-biang-keroknya)</t>
+        </is>
+      </c>
+      <c r="E161" s="6" t="inlineStr">
+        <is>
+          <t>NEGATIF</t>
+        </is>
+      </c>
+      <c r="F161" s="6" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="G161" s="6" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B162" s="6" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C162" s="6" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D162" s="7" t="inlineStr">
+        <is>
+          <t>[Dilanda Panas Ekstrem, Warga Eropa Panic Buying Rebutan AC](https://finance.detik.com/berita-ekonomi-bisnis/d-8550247/dilanda-panas-ekstrem-warga-eropa-panic-buying-rebutan-ac)</t>
+        </is>
+      </c>
+      <c r="E162" s="6" t="inlineStr">
+        <is>
+          <t>NEGATIF</t>
+        </is>
+      </c>
+      <c r="F162" s="6" t="n">
+        <v>-0.511</v>
+      </c>
+      <c r="G162" s="6" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="inlineStr">
+        <is>
+          <t>[Terungkap Biang Kerok AS Serang Iran Lagi](https://finance.detik.com/berita-ekonomi-bisnis/d-8550246/terungkap-biang-kerok-as-serang-iran-lagi)</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="inlineStr">
+        <is>
+          <t>[Purbaya soal Efisiensi Anggaran MBG: Saya Maunya Nol, Tapi Nggak Bisa Kan](https://finance.detik.com/berita-ekonomi-bisnis/d-8549550/purbaya-soal-efisiensi-anggaran-mbg-saya-maunya-nol-tapi-nggak-bisa-kan)</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="inlineStr">
+        <is>
+          <t>[Prabowo Singgung Swasta Ikut Nikmati Susbidi Listrik-BBM](https://finance.detik.com/berita-ekonomi-bisnis/d-8550638/prabowo-singgung-swasta-ikut-nikmati-susbidi-listrik-bbm)</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D166" s="3" t="inlineStr">
+        <is>
+          <t>[Dapat Usulan Untung BUMN buat Biaya Riset, Prabowo: Masalahnya Ada Laba Nggak?](https://finance.detik.com/berita-ekonomi-bisnis/d-8550603/dapat-usulan-untung-bumn-buat-biaya-riset-prabowo-masalahnya-ada-laba-nggak)</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B167" s="4" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C167" s="4" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>[Prabowo Singgung soal Gaduh-gaduh: Kapan Rakyat Sejahtera?](https://finance.detik.com/berita-ekonomi-bisnis/d-8548940/prabowo-singgung-soal-gaduh-gaduh-kapan-rakyat-sejahtera)</t>
+        </is>
+      </c>
+      <c r="E167" s="4" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="F167" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G167" s="4" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="inlineStr">
+        <is>
+          <t>[Beras IR. III (IR 64)](https://finance.detik.com/info-pangan/jakarta/beras-ir-iii-ir-64)</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr">
+        <is>
+          <t>[Cabe Merah Keriting](https://finance.detik.com/info-pangan/jakarta/cabe-merah-keriting)</t>
+        </is>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="inlineStr">
+        <is>
+          <t>[Daging Sapi Murni (Semur)](https://finance.detik.com/info-pangan/jakarta/daging-sapi-murni-semur)</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="inlineStr">
+        <is>
+          <t>[DJP Tunjuk 7 Pemungut Pajak Digital Baru, Ada Strava](https://finance.detik.com/berita-ekonomi-bisnis/d-8550575/djp-tunjuk-7-pemungut-pajak-digital-baru-ada-strava)</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="inlineStr">
+        <is>
+          <t>[Alat Makan &amp; Minum Diskon Gede-gedean di Transmart Full Day Sale](https://finance.detik.com/berita-ekonomi-bisnis/d-8550477/alat-makan-minum-diskon-gede-gedean-di-transmart-full-day-sale)</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t>[Pemerintah Kantongi Rp 52,85 T dari Pajak Kripto-Pinjol, Ini Rinciannya](https://finance.detik.com/berita-ekonomi-bisnis/d-8550537/pemerintah-kantongi-rp-52-85-t-dari-pajak-kripto-pinjol-ini-rinciannya)</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="inlineStr">
+        <is>
+          <t>Rekomendasi untuk Anda</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
         <is>
           <t>detik finance</t>
         </is>
@@ -6150,7 +6710,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
@@ -6165,11 +6725,11 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
@@ -6180,11 +6740,11 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
@@ -6195,11 +6755,11 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>72.0%</t>
+          <t>72.3%</t>
         </is>
       </c>
     </row>
@@ -6210,7 +6770,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>-0.063</v>
+        <v>-0.065</v>
       </c>
       <c r="C6" s="8" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Fix audit: emas column mapping, sentimen noise filter, pertanian article filter, crypto market cap display
</commit_message>
<xml_diff>
--- a/data/sentimen_berita.xlsx
+++ b/data/sentimen_berita.xlsx
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G174"/>
+  <dimension ref="A1:G190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6662,6 +6662,566 @@
         <v>0</v>
       </c>
       <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr">
+        <is>
+          <t>detikFinance - Berita Ekonomi Bisnis, dan Investasi Hari Ini</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B176" s="6" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C176" s="6" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D176" s="7" t="inlineStr">
+        <is>
+          <t>[Harga Emas Antam Turun dalam Sepekan, Buyback Anjlok Rp 20 Ribu/Gram](https://finance.detik.com/berita-ekonomi-bisnis/d-8550494/harga-emas-antam-turun-dalam-sepekan-buyback-anjlok-rp-20-ribu-gram)</t>
+        </is>
+      </c>
+      <c r="E176" s="6" t="inlineStr">
+        <is>
+          <t>NEGATIF</t>
+        </is>
+      </c>
+      <c r="F176" s="6" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="G176" s="6" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B177" s="6" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C177" s="6" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D177" s="7" t="inlineStr">
+        <is>
+          <t>[Harga Ayam di Pasar Ikut Anjlok Jadi Rp 35.000/Kg, Ini Biang Keroknya](https://finance.detik.com/berita-ekonomi-bisnis/d-8550248/harga-ayam-di-pasar-ikut-anjlok-jadi-rp-35-000-kg-ini-biang-keroknya)</t>
+        </is>
+      </c>
+      <c r="E177" s="6" t="inlineStr">
+        <is>
+          <t>NEGATIF</t>
+        </is>
+      </c>
+      <c r="F177" s="6" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="G177" s="6" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B178" s="6" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C178" s="6" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D178" s="7" t="inlineStr">
+        <is>
+          <t>[Dilanda Panas Ekstrem, Warga Eropa Panic Buying Rebutan AC](https://finance.detik.com/berita-ekonomi-bisnis/d-8550247/dilanda-panas-ekstrem-warga-eropa-panic-buying-rebutan-ac)</t>
+        </is>
+      </c>
+      <c r="E178" s="6" t="inlineStr">
+        <is>
+          <t>NEGATIF</t>
+        </is>
+      </c>
+      <c r="F178" s="6" t="n">
+        <v>-0.511</v>
+      </c>
+      <c r="G178" s="6" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>[Terungkap Biang Kerok AS Serang Iran Lagi](https://finance.detik.com/berita-ekonomi-bisnis/d-8550246/terungkap-biang-kerok-as-serang-iran-lagi)</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D180" s="3" t="inlineStr">
+        <is>
+          <t>[Purbaya soal Efisiensi Anggaran MBG: Saya Maunya Nol, Tapi Nggak Bisa Kan](https://finance.detik.com/berita-ekonomi-bisnis/d-8549550/purbaya-soal-efisiensi-anggaran-mbg-saya-maunya-nol-tapi-nggak-bisa-kan)</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>[Prabowo Singgung Swasta Ikut Nikmati Susbidi Listrik-BBM](https://finance.detik.com/berita-ekonomi-bisnis/d-8550638/prabowo-singgung-swasta-ikut-nikmati-susbidi-listrik-bbm)</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D182" s="3" t="inlineStr">
+        <is>
+          <t>[Dapat Usulan Untung BUMN buat Biaya Riset, Prabowo: Masalahnya Ada Laba Nggak?](https://finance.detik.com/berita-ekonomi-bisnis/d-8550603/dapat-usulan-untung-bumn-buat-biaya-riset-prabowo-masalahnya-ada-laba-nggak)</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C183" s="4" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D183" s="5" t="inlineStr">
+        <is>
+          <t>[Prabowo Singgung soal Gaduh-gaduh: Kapan Rakyat Sejahtera?](https://finance.detik.com/berita-ekonomi-bisnis/d-8548940/prabowo-singgung-soal-gaduh-gaduh-kapan-rakyat-sejahtera)</t>
+        </is>
+      </c>
+      <c r="E183" s="4" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="F183" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G183" s="4" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="inlineStr">
+        <is>
+          <t>[Beras IR. III (IR 64)](https://finance.detik.com/info-pangan/jakarta/beras-ir-iii-ir-64)</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>[Cabe Merah Keriting](https://finance.detik.com/info-pangan/jakarta/cabe-merah-keriting)</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>[Daging Sapi Murni (Semur)](https://finance.detik.com/info-pangan/jakarta/daging-sapi-murni-semur)</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D187" s="3" t="inlineStr">
+        <is>
+          <t>[DJP Tunjuk 7 Pemungut Pajak Digital Baru, Ada Strava](https://finance.detik.com/berita-ekonomi-bisnis/d-8550575/djp-tunjuk-7-pemungut-pajak-digital-baru-ada-strava)</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="inlineStr">
+        <is>
+          <t>[Pemerintah Kantongi Rp 52,85 T dari Pajak Kripto-Pinjol, Ini Rinciannya](https://finance.detik.com/berita-ekonomi-bisnis/d-8550537/pemerintah-kantongi-rp-52-85-t-dari-pajak-kripto-pinjol-ini-rinciannya)</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>[Rak Besi Banting Harga di Transmart Full Day Sale, Serbu!](https://finance.detik.com/berita-ekonomi-bisnis/d-8550451/rak-besi-banting-harga-di-transmart-full-day-sale-serbu)</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>detik finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>berita ekonomi</t>
+        </is>
+      </c>
+      <c r="D190" s="3" t="inlineStr">
+        <is>
+          <t>[PLTP Dieng Unit 2 Mulai Dibangun, Segini Kapasitasnya](https://finance.detik.com/energi/d-8550378/pltp-dieng-unit-2-mulai-dibangun-segini-kapasitasnya)</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
         <is>
           <t>detik finance</t>
         </is>
@@ -6710,7 +7270,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
@@ -6725,11 +7285,11 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
@@ -6740,11 +7300,11 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
@@ -6755,11 +7315,11 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>72.3%</t>
+          <t>72.5%</t>
         </is>
       </c>
     </row>
@@ -6770,7 +7330,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>-0.065</v>
+        <v>-0.067</v>
       </c>
       <c r="C6" s="8" t="inlineStr"/>
     </row>

</xml_diff>